<commit_message>
docs: rewrite copy to read as original work, drop AI-tool convention files
Trimmed narrated self-correction commentary from code comments and
docstrings (the "originally X, changed to Y because..." style) down to
plain statements of the final assumption. Removed references to
internal file/tool conventions that had leaked into the actual
deliverables (Excel tab subtitles, data sources table).

Rewrote the README: dropped the "Interview Talking Points" section
entirely and the skills-demonstrated bullet dump, rewrote Key Findings
as prose instead of a bulleted report summary, varied repeated stock
phrasing across the README/dashboard/metadata.

Untracked CLAUDE.md, frontend/CLAUDE.md, and frontend/AGENTS.md from
git (kept locally, now gitignored) -- these are AI-coding-tool
convention files with no reason to be in a public repo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/scoring_model.xlsx
+++ b/outputs/scoring_model.xlsx
@@ -819,7 +819,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Thresholds recalibrated against real 5-city data ranges where the original placeholder bands did not discriminate (see analysis/scoring_model.py docstring)</t>
+          <t>Thresholds set against the real range of values across the 5 candidate metros</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>5yr appreciation (RECALIBRATED): &gt;25%</t>
+          <t>5yr appreciation: &gt;25%</t>
         </is>
       </c>
       <c r="B37" s="12" t="inlineStr">
@@ -1303,7 +1303,7 @@
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>Dimension 4 — Competitive Saturation (weight 20%, INVERTED, RECALIBRATED)</t>
+          <t>Dimension 4 — Competitive Saturation (weight 20%, INVERTED)</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>Dimension 5 — Retail Lease Rate (weight 10%, INVERTED, RECALIBRATED)</t>
+          <t>Dimension 5 — Retail Lease Rate (weight 10%, INVERTED)</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Baseline: weights as specified in CLAUDE.md (Pop&amp;Growth 15%, Income&amp;Spend 20%, Housing 20%, Competition 20%, Lease 10%, Labor 10%, Logistics 5%)</t>
+          <t>Baseline: Pop&amp;Growth 15%, Income&amp;Spend 20%, Housing 20%, Competition 20%, Lease 10%, Labor 10%, Logistics 5%</t>
         </is>
       </c>
     </row>
@@ -2690,12 +2690,12 @@
       </c>
       <c r="C14" s="21" t="inlineStr">
         <is>
-          <t>Project team assumptions, recalibrated against real specialty-retail staffing/conversion benchmarks</t>
+          <t>Project team assumptions, benchmarked against specialty-retail staffing and conversion norms</t>
         </is>
       </c>
       <c r="D14" s="21" t="inlineStr">
         <is>
-          <t>See CLAUDE.md</t>
+          <t>See README.md</t>
         </is>
       </c>
       <c r="E14" s="21" t="inlineStr">

</xml_diff>